<commit_message>
add a visualization and evaluation in the main code
</commit_message>
<xml_diff>
--- a/ds-lab2/main/courses_with_no_relevant_skill_roles.xlsx
+++ b/ds-lab2/main/courses_with_no_relevant_skill_roles.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A313"/>
+  <dimension ref="A1:A316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,1996 +501,1996 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Biometric Systems</t>
+          <t>Advanced Information Security</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Cryptanalysis</t>
+          <t>Biometric Systems</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cryptographic Engineering</t>
+          <t>Application of Machine Learning in Information Security</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cryptographic protocols</t>
+          <t>Cryptanalysis</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mathematical Logic for Computer Science</t>
+          <t>Cryptographic Engineering</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Advanced algebraic structures</t>
+          <t>Cryptographic protocols</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Advanced coding algorithms</t>
+          <t>Mathematical Logic for Computer Science</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Applied Information Theory</t>
+          <t>Advanced algebraic structures</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Random processes</t>
+          <t>Advanced coding algorithms</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Open-Source Intelligence</t>
+          <t>Applied Information Theory</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Machine Learning</t>
+          <t>Random processes</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Access and Transport Networks</t>
+          <t>Open-Source Intelligence</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Dependability and Performance with Discrete Event Simulation</t>
+          <t>Machine Learning</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Advanced Network Control and Management</t>
+          <t>Access and Transport Networks</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Applied Project Management</t>
+          <t>Dependability and Performance with Discrete Event Simulation</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Applied Cryptography and Network Security</t>
+          <t>Advanced Network Control and Management</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Intrusion Detection in Physical and Virtual Networks</t>
+          <t>Finance for Science and Technology Students</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Introduction to Data Privacy</t>
+          <t>Applied Project Management</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Dependable Performance Design</t>
+          <t>Applied Cryptography and Network Security</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Design of Cyber-Physical Systems</t>
+          <t>Intrusion Detection in Physical and Virtual Networks</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Advanced Internet Technologies - Networked Systems, Specialization Course</t>
+          <t>Introduction to Data Privacy</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Distributed Systems</t>
+          <t>Dependable Performance Design</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Quantum Cryptography</t>
+          <t>Design of Cyber-Physical Systems</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Time Series Analysis</t>
+          <t>Advanced Internet Technologies - Networked Systems, Specialization Course</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Performance analysis of computer systems</t>
+          <t>Distributed Systems</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>From an Idea to Reality</t>
+          <t>Quantum Cryptography</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Network Measurements and Analysis</t>
+          <t>Time Series Analysis</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Machine Learning</t>
+          <t>Performance analysis of computer systems</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Machine Learning for Earth Observation powered by Supercomputers</t>
+          <t>From an Idea to Reality</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Programming Projects on Internet of Things</t>
+          <t>Network Measurements and Analysis</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Introduction to deep neural networks</t>
+          <t>Machine Learning</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>Machine Learning for Earth Observation powered by Supercomputers</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Software Testing</t>
+          <t>Programming Projects on Internet of Things</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Fundaments of the Internet</t>
+          <t>Introduction to deep neural networks</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Reasoned Programming</t>
+          <t>Applied Cryptography</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Biometric security systems</t>
+          <t>Software Testing</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Foreign language in science and technology</t>
+          <t>Fundaments of the Internet</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Introduction to cryptography</t>
+          <t>Reasoned Programming</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Fighting crime in cyberspace and legal aspects of cybersecurity</t>
+          <t>Biometric security systems</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Security of IoT systems</t>
+          <t>Foreign language in science and technology</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Security and safety in control systems and industrial networks</t>
+          <t>Introduction to cryptography</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>History of ideas and scientific discoveries</t>
+          <t>Fighting crime in cyberspace and legal aspects of cybersecurity</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Quantum cryptography</t>
+          <t>Security of IoT systems</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Mathematical foundations of cryptography</t>
+          <t>Security and safety in control systems and industrial networks</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Information society</t>
+          <t>History of ideas and scientific discoveries</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Cryptography and Network Security</t>
+          <t>Quantum cryptography</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Digital Signal Processing for Communications and Information Systems</t>
+          <t>Mathematical foundations of cryptography</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Analog and Mixed-Signal Electronics for Signal Processing</t>
+          <t>Information society</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Analysis of Digital Communication Systems</t>
+          <t>Cryptography and Network Security</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Building Blocks for Telecom Systems</t>
+          <t>Digital Signal Processing for Communications and Information Systems</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Design of Digital Platforms</t>
+          <t>Analog and Mixed-Signal Electronics for Signal Processing</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Computer Architectures</t>
+          <t>Analysis of Digital Communication Systems</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Stochastic Signal and System Analysis</t>
+          <t>Building Blocks for Telecom Systems</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Electromagnetic Propagation</t>
+          <t>Design of Digital Platforms</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Mobile Networks</t>
+          <t>Computer Architectures</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>P&amp;D ICT Security and Networks</t>
+          <t>Stochastic Signal and System Analysis</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Hardware Security</t>
+          <t>Electromagnetic Propagation</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Telecommunications and Security Management</t>
+          <t>Mobile Networks</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Privacy Technologies</t>
+          <t>Hardware Security</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>e-Security</t>
+          <t>Telecommunications and Security Management</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Software for Real-Time Control</t>
+          <t>Privacy Technologies</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>6G Communication Networks</t>
+          <t>e-Security</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Distributed Systems</t>
+          <t>Software for Real-Time Control</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Advanced Methods in Cryptography</t>
+          <t>6G Communication Networks</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Image Analysis and Understanding</t>
+          <t>Distributed Systems</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Satellite Navigation and Communications</t>
+          <t>Advanced Methods in Cryptography</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Multimedia Technology and Coding</t>
+          <t>Image Analysis and Understanding</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Computer Algebra for Cryptography</t>
+          <t>Satellite Navigation and Communications</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Philosophy of Technology</t>
+          <t>Multimedia Technology and Coding</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Engineering Economy</t>
+          <t>Philosophy of Technology</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Introduction to Safety Engineering</t>
+          <t>Engineering Economy</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Total Quality Management</t>
+          <t>Introduction to Safety Engineering</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Intellectual Property Management</t>
+          <t>Total Quality Management</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>New and Emerging Technologies</t>
+          <t>Intellectual Property Management</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Robotics Applications</t>
+          <t>New and Emerging Technologies</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Data Science Applications II</t>
+          <t>Robotics Applications</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Basic General Algebra</t>
+          <t>Data Science Applications II</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Basic algorithms</t>
+          <t>Basic General Algebra</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Information theory</t>
+          <t>Basic algorithms</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Correcting codes</t>
+          <t>Information theory</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Complexity</t>
+          <t>Correcting codes</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Complexity</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Cryptanalysis</t>
+          <t>Cryptography</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Software Security</t>
+          <t>Elliptic Curves for Cryptography</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Euclidean networks in cryptography</t>
+          <t>Cryptanalysis</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Blockchain principles and applications</t>
+          <t>Software Security</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Protocol Security</t>
+          <t>Euclidean networks in cryptography</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Correcting codes in cryptography</t>
+          <t>Blockchain principles and applications</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Quantum Cryptography</t>
+          <t>Parallel programming, GPU</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Algorithmic number theory for cryptography</t>
+          <t>Protocol Security</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Big Data Infrastructures</t>
+          <t>Correcting codes in cryptography</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Quantum Cryptography</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Basic Network Security</t>
+          <t>Algorithmic number theory for cryptography</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>Big Data Infrastructures</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Machine Learning &amp; AI for Security</t>
+          <t>Cryptography</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Mobile Network Security</t>
+          <t>Basic Network Security</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Embedded Security Assessment</t>
+          <t>Applied Cryptography</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cryptology </t>
+          <t>Machine Learning &amp; AI for Security</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Principles of data protection</t>
+          <t>Mobile Network Security</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Advanced Network Security</t>
+          <t>Embedded Security Assessment</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Physical aspects of digital security</t>
+          <t xml:space="preserve">Cryptology </t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Verification of security protocols</t>
+          <t>Cyberattacks Crime and Defenses</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Cryptographic protocols</t>
+          <t>Advanced Network Security</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Applied cryptography</t>
+          <t>Physical aspects of digital security</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Advanced algorithms</t>
+          <t>Verification of security protocols</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Intrusion Detection Laboratory</t>
+          <t>Cryptographic protocols</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>CRYPTOGRAPHY</t>
+          <t>Applied cryptography</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>DEEP LEARNING FUNDAMENTALS</t>
+          <t>Advanced algorithms</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>MACHINE LEARNING APPLIED TO CYBERSECURITY AND CYBERCRIME</t>
+          <t>Intrusion Detection Laboratory</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>AUTHENTICATION TECHNOLOGIES</t>
+          <t>CRYPTOGRAPHY</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Algorithms &amp; Data Structures</t>
+          <t>DEEP LEARNING FUNDAMENTALS</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>MACHINE LEARNING APPLIED TO CYBERSECURITY AND CYBERCRIME</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Discrete mathematics</t>
+          <t>AUTHENTICATION TECHNOLOGIES</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Cryptology &amp; Applications</t>
+          <t>Algorithms &amp; Data Structures</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Networking I</t>
+          <t>Analysis</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>5G Mobile Networks, Technologies &amp; Security</t>
+          <t>Discrete mathematics</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Network Defense &amp; Architecture</t>
+          <t>Cryptology &amp; Applications</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Information systems security</t>
+          <t>Networking I</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Networks &amp; Cloud Technologies and Security (Computer networks and cloud technologies)</t>
+          <t>object oriented programing</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Operating System &amp; Architecture</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Hardware &amp; Wireless Security (Hardware and embedded security)</t>
+          <t>5G Mobile Networks, Technologies &amp; Security</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Hardware &amp; Wireless Security (Wireless and device-to-device communication Security)</t>
+          <t>Network Defense &amp; Architecture</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Web Applications</t>
+          <t>Networks &amp; Cloud Technologies and Security (Computer networks and cloud technologies)</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Advanced cryptography</t>
+          <t>Networks &amp; Cloud Technologies and Security (Network and Cloud Security)</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>AI and Cybersecurity</t>
+          <t>Cryptography</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Data protection, Privacy and Anonymity</t>
+          <t>Hardware &amp; Wireless Security (Hardware and embedded security)</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Technology and Innovation Management in Cybersecurity</t>
+          <t>Hardware &amp; Wireless Security (Wireless and device-to-device communication Security)</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Post-Quantum Cryptography</t>
+          <t>Web Applications</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Network design - Introduction</t>
+          <t>Advanced cryptography</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>System administration - Introduction</t>
+          <t>AI and Cybersecurity</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Network design - Switching and Routing</t>
+          <t>Data protection, Privacy and Anonymity</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Network design - WAN and operator networks</t>
+          <t>Post-Quantum Cryptography</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Network security</t>
+          <t>Network design - Introduction</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Network design - Wireless networks</t>
+          <t>System administration - Introduction</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>System administration - Databases</t>
+          <t>Network design - Switching and Routing</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>AUTOMATED REASONING</t>
+          <t>Network design - WAN and operator networks</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>DEEP LEARNING</t>
+          <t>Network security</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>VERIFICATION AND VALIDATION TECHNIQUES IN AI AND CYBERSECURITY</t>
+          <t>Network design - Wireless networks</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>ADVANCED DATA SCIENCE</t>
+          <t>Script programming</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>ADVANCED DATABASE SYSTEMS</t>
+          <t>System administration - Databases</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>AUDITORY AND TACTILE INTERACTIONS</t>
+          <t>AUTOMATED REASONING</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>COMPUTER VISION</t>
+          <t>DEEP LEARNING</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>DISTRIBUTED SYSTEMS</t>
+          <t>VERIFICATION AND VALIDATION TECHNIQUES IN AI AND CYBERSECURITY</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>FORMAL METHODS FOR SECURITY</t>
+          <t>ADVANCED ALGORITHMS</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>FOUNDATIONS OF NEURAL NETWORKS</t>
+          <t>ADVANCED DATA SCIENCE</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>INFORMATION RETRIEVAL</t>
+          <t>ADVANCED DATABASE SYSTEMS</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>QUANTUM COMPUTING AND COMMUNICATION</t>
+          <t>AUDITORY AND TACTILE INTERACTIONS</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Communication Technology</t>
+          <t>COMPUTER VISION</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Computers and Programming 1</t>
+          <t>DISTRIBUTED SYSTEMS</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Legal Theory</t>
+          <t>FORMAL METHODS FOR SECURITY</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Foundations of Cryptography</t>
+          <t>FOUNDATIONS OF NEURAL NETWORKS</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>GENERATIVE AI</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Computers and Programming 2</t>
+          <t>INFORMATION RETRIEVAL</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Fundamentals of Information and Communication Technologies</t>
+          <t>QUANTUM COMPUTING AND COMMUNICATION</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Data Communication</t>
+          <t>Communication Technology</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Theoretical Informatics</t>
+          <t>Computers and Programming 1</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>ICT Security 2</t>
+          <t>Legal Theory</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Multimedia Services</t>
+          <t>Foundations of Cryptography</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Electrical Engineering 1</t>
+          <t>Applied Cryptography</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Access and Transport Networks</t>
+          <t>Computers and Programming 2</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Security Systems</t>
+          <t>Fundamentals of Information and Communication Technologies</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Introduction to Computer Typography and Graphics</t>
+          <t>Data Communication</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Network Architecture</t>
+          <t>Theoretical Informatics</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Digital Electronics 1</t>
+          <t>ICT Security 2</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Hardware of Computer Networks</t>
+          <t>Multimedia Services</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Communication Systems for IoT</t>
+          <t>Electrical Engineering 1</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Mobile Communication</t>
+          <t>Access and Transport Networks</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Object-Oriented Programming</t>
+          <t>Security Systems</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Transmission Media</t>
+          <t>Introduction to Computer Typography and Graphics</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>The C++ Programming Language</t>
+          <t>Network Architecture</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Analog Technology</t>
+          <t>Digital Electronics 1</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Automobile Electric and Electronic Systems</t>
+          <t>Hardware of Computer Networks</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Computer Modeling of Electrical Devices and Components</t>
+          <t>Communication Systems for IoT</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Television Technology and Multimedia</t>
+          <t>Mobile Communication</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Artificial Intelligence</t>
+          <t>Object-Oriented Programming</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Introduction to Programming Systems</t>
+          <t>Transmission Media</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Data Science</t>
+          <t>The C++ Programming Language</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Network Security</t>
+          <t>Analog Technology</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Privacy &amp; Cryptography</t>
+          <t>Automobile Electric and Electronic Systems</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>Computer Modeling of Electrical Devices and Components</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Network Security</t>
+          <t>Television Technology and Multimedia</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Malware Analysis</t>
+          <t>Artificial Intelligence</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Cryptography and Network Security</t>
+          <t>Introduction to Programming Systems</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Cryptographic Protocols</t>
+          <t>Data Science</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Advanced Methods in Cryptography</t>
+          <t>Privacy &amp; Cryptography</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Privacy Technologies</t>
+          <t>Applied Cryptography</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Advanced Privacy Technologies</t>
+          <t>Network Security</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Design of Digital Platforms</t>
+          <t>Malware Analysis</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Design Seminar for Digital Platforms</t>
+          <t>Cryptography and Network Security</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Hardware Security</t>
+          <t>Cryptographic Protocols</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Development of Secure Software</t>
+          <t>Advanced Methods in Cryptography</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Security and Privacy in Contemporary Distributed Software Systems</t>
+          <t>Privacy Technologies</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Practical Cryptography</t>
+          <t>Advanced Privacy Technologies</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>Design of Digital Platforms</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Security and Applications in Trusted Hardware</t>
+          <t>Design Seminar for Digital Platforms</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Fraud Detection</t>
+          <t>Hardware Security</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Processing of Structured Documents</t>
+          <t>Development of Secure Software</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Big Data and Cloud Computing</t>
+          <t>Security and Privacy in Contemporary Distributed Software Systems</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Advanced Topics in Databases</t>
+          <t>Practical Cryptography</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Advanced Topics in Networking</t>
+          <t>Applied Cryptography</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Network Security</t>
+          <t>Fraud Detection</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
+          <t>Processing of Structured Documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Big Data and Cloud Computing</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Advanced Topics in Databases</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Advanced Topics in Networking</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Network Security</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
           <t xml:space="preserve">Data security and protection
 </t>
         </is>
       </c>
     </row>
-    <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>Component Security</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>FAULT DIAGNOSIS AND ESTIMATION IN DYNAMICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>INDUSTRIAL SOFTWARE DEVELOPMENT</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>MACHINE LEARNING</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>ARTIFICIAL INTELLIGENCE</t>
-        </is>
-      </c>
-    </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>OPERATING SYSTEMS</t>
+          <t>FAULT DIAGNOSIS AND ESTIMATION IN DYNAMICAL</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>SUPERVISORY CONTROL AND MONITORING</t>
+          <t>INDUSTRIAL SOFTWARE DEVELOPMENT</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>DATA DRIVEN MODELS FOR SYSTEM ENGINEERING</t>
+          <t>MACHINE LEARNING</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>CRITICAL INFRASTRUCTURES FOR INNOVATIVE POWER DISTRIBUTION</t>
+          <t>ARTIFICIAL INTELLIGENCE</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>MEASUREMENTS AND CYBERSECURITY FOR SMART GRID</t>
+          <t>OPERATING SYSTEMS</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>INTERNET OF THINGS</t>
+          <t>SUPERVISORY CONTROL AND MONITORING</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>ADVANCED EMBEDDED SYSTEMS</t>
+          <t>DATA DRIVEN MODELS FOR SYSTEM ENGINEERING</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>NETWORKED CONTROL SYSTEMS AND SECURITY</t>
+          <t>CRITICAL INFRASTRUCTURES FOR INNOVATIVE POWER DISTRIBUTION</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>STOCHASTIC MODELS</t>
+          <t>INTERNET OF THINGS</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>PHYSICAL-LAYER TECHNIQUES FOR WIRELESS COMMUNICATION SECURITY</t>
+          <t>ADVANCED EMBEDDED SYSTEMS</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>BIOMETRIC TECHNOLOGIES AND BEHAVIOURAL SECURITY</t>
+          <t>NETWORKED CONTROL SYSTEMS AND SECURITY</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Secure Communications</t>
+          <t>STOCHASTIC MODELS</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Laboratory of security and applied cryptography</t>
+          <t>PHYSICAL-LAYER TECHNIQUES FOR WIRELESS COMMUNICATION SECURITY</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Security Technologies</t>
+          <t>BIOMETRIC TECHNOLOGIES AND BEHAVIOURAL SECURITY</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Advanced Topics in Information Technology Security</t>
+          <t>Secure Communications</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Machine learning and natural language processing</t>
+          <t>Software Reverse Engineering</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Machine Learning in Image Processing</t>
+          <t>Laboratory of security and applied cryptography</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>System Development in C#/.NET</t>
+          <t>Security Technologies</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>GPU Programming</t>
+          <t>Advanced Topics in Information Technology Security</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Python Seminar</t>
+          <t>Machine learning and natural language processing</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Introduction to Quantum Computer Programming</t>
+          <t>Machine Learning in Image Processing</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Introduction to IoT</t>
+          <t>System Development in C#/.NET</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>GPU Programming</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Fundaments of Cryptography</t>
+          <t>Python Seminar</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Probability in Computer Science</t>
+          <t>Introduction to Quantum Computer Programming</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Advanced Computer Networking</t>
+          <t>Introduction to IoT</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Statistics for Computer Science</t>
+          <t>Python</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t xml:space="preserve">Formal Methods for Software Analysis </t>
+          <t>Fundaments of Cryptography</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Advanced Topics in Information Technology Security</t>
+          <t>Probability in Computer Science</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Mathematical Foundations of Computer Science</t>
+          <t>Advanced Computer Networking</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Foundations of Programming</t>
+          <t>Statistics for Computer Science</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Computer Systems</t>
+          <t xml:space="preserve">Formal Methods for Software Analysis </t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Database Systems</t>
+          <t>Advanced Topics in Information Technology Security</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Introduction to DB and IS</t>
+          <t>Mathematical Foundations of Computer Science</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Introduction to Programming and Algorithms II</t>
+          <t>Foundations of Programming</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Principles of low-level programming</t>
+          <t>Computer Systems</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>Database Systems</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Computer Networks</t>
+          <t>Introduction to Programming and Algorithms II</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>Computer Networks - practicals</t>
+          <t>Principles of low-level programming</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>UNIX</t>
+          <t>Operating Systems</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>ICT Law II</t>
+          <t>Computer Networks</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Cyber Warfare</t>
+          <t>Computer Networks - practicals</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Introduction to Informatics</t>
+          <t>UNIX</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Pros and Cons of Intelligent Systems</t>
+          <t>ICT Law II</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Linear algebra and discrete mathematics</t>
+          <t>Cyber Warfare</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Foundations of Object Oriented Programming in Java</t>
+          <t>Introduction to Informatics</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Registration for SB200</t>
+          <t>Pros and Cons of Intelligent Systems</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Applied Information Systems</t>
+          <t>Linear algebra and discrete mathematics</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Authentication and Access Control</t>
+          <t>Foundations of Object Oriented Programming in Java</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Electronic Document Preparation</t>
+          <t>Registration for SB200</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>Authentication and Access Control</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Foundations of Cryptography</t>
+          <t>Electronic Document Preparation</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Cyber-Physical Security in Time-Critical Systems</t>
+          <t>Applied Cryptography</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Design of Fault-tolerant Systems</t>
+          <t>Foundations of Cryptography</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Hardware Security</t>
+          <t>Cyber-Physical Security in Time-Critical Systems</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Foundations of Machine Learning</t>
+          <t>Design of Fault-tolerant Systems</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Machine Learning</t>
+          <t>Hardware Security</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Machine Learning, Advanced Course</t>
+          <t>Foundations of Machine Learning</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Artificial Neural Networks and Deep Architectures</t>
+          <t>Machine Learning</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Advanced Algorithms</t>
+          <t>Machine Learning, Advanced Course</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Parallel and Distributed Computing</t>
+          <t>Artificial Neural Networks and Deep Architectures</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Statistical Methods in Applied Computer Science</t>
+          <t>Advanced Algorithms</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Interaction Design Methods</t>
+          <t>Parallel and Distributed Computing</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Reinforcement Learning</t>
+          <t>Statistical Methods in Applied Computer Science</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Degree Project in Computer Science and Engineering, specialising in Cybersecurity</t>
+          <t>Reinforcement Learning</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Software Safety and Security</t>
+          <t>Degree Project in Computer Science and Engineering, specialising in Cybersecurity</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>Software Safety and Security</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Biometrics</t>
+          <t>Applied Cryptography</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Machine Learning Applied to Security</t>
+          <t>Biometrics</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Identification, Authentication and Authorization</t>
+          <t>Machine Learning Applied to Security</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Quantum Security</t>
+          <t>Identification, Authentication and Authorization</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Information Technology Security Methods</t>
+          <t>Quantum Security</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Cryptographic Systems</t>
+          <t>Information Technology Security Methods</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Malware Analysis Methods</t>
+          <t>Cryptographic Systems</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>FOUNDATIONS OF LEGAL SYSTEM AND STATE ORGANISATION</t>
+          <t>Malware Analysis Methods</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>NATIONAL SECURITY SYSTEM</t>
+          <t>FOUNDATIONS OF LEGAL SYSTEM AND STATE ORGANISATION</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>INTRODUCTION TO SOFTWARE DEVELOPMENT</t>
+          <t>NATIONAL SECURITY SYSTEM</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>PSYCHOLOGY IN CRIMINAL JUSTICE</t>
+          <t>INTRODUCTION TO SOFTWARE DEVELOPMENT</t>
         </is>
       </c>
     </row>
@@ -2553,68 +2553,89 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Data Analytics and Machine Learning</t>
+          <t>Network and Communications Security</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>Data Analytics and Machine Learning</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Advanced Cryptographic and Security Technologies (Blockchain technologies)</t>
+          <t>Applied Cryptography</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Aplicated math</t>
+          <t>Advanced Cryptographic and Security Technologies (Blockchain technologies)</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Operating Systems and Virtualization</t>
+          <t>Programming fundamentals</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Algorithms and Data Structures</t>
+          <t>Aplicated math</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Applied Mathematics Complements</t>
+          <t>Operating Systems and Virtualization</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Introduction to Computer Networks</t>
+          <t>Algorithms and Data Structures</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Introduction to Design Thinking</t>
+          <t>Applied Mathematics Complements</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
+        <is>
+          <t>Introduction to Computer Networks</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Introduction to Design Thinking</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Statistics and Probabilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
         <is>
           <t>Applied Cryptography</t>
         </is>

</xml_diff>

<commit_message>
update and save for not relavance course-skill
</commit_message>
<xml_diff>
--- a/ds-lab2/main/courses_with_no_relevant_skill_roles.xlsx
+++ b/ds-lab2/main/courses_with_no_relevant_skill_roles.xlsx
@@ -425,41 +425,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A316"/>
+  <dimension ref="A1:A289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Course Title</t>
+          <t>Not Relevant Course Titles</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Introduction to Data Science Tools</t>
+          <t>GENERATIVE AI</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Research Methods and Scientific Ethics</t>
+          <t>Principles of low-level programming</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Computer Networks and Security</t>
+          <t>Computers and Programming 2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Operating Systems and System Programming</t>
+          <t>Fighting crime in cyberspace and legal aspects of cybersecurity</t>
         </is>
       </c>
     </row>
@@ -473,2171 +473,1982 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>German/Macedonian</t>
+          <t>Privacy Technologies</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Scripting Languages</t>
+          <t>Robotics Applications</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>Applied Cryptography and Network Security</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Coding Theory and Applications</t>
+          <t>CRIMINAL JUSTICE AND SECURITY TERMINOLOGY IN ENGLISH</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Advanced Information Security</t>
+          <t>Advanced coding algorithms</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Biometric Systems</t>
+          <t>Cryptographic protocols</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Application of Machine Learning in Information Security</t>
+          <t>Advanced Topics in Information Technology Security</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Cryptanalysis</t>
+          <t>Practical Cryptography</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cryptographic Engineering</t>
+          <t>Introduction to Informatics</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Cryptographic protocols</t>
+          <t>COMPUTER VISION</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mathematical Logic for Computer Science</t>
+          <t>Programming Projects on Internet of Things</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Advanced algebraic structures</t>
+          <t>Introduction to Programming and Algorithms II</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Advanced coding algorithms</t>
+          <t>Linear algebra and discrete mathematics</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Applied Information Theory</t>
+          <t>Probability in Computer Science</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Random processes</t>
+          <t>Foundations of Cryptography</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Open-Source Intelligence</t>
+          <t>Parallel and Distributed Computing</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Machine Learning</t>
+          <t>Advanced Privacy Technologies</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Access and Transport Networks</t>
+          <t>Quantum Security</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Dependability and Performance with Discrete Event Simulation</t>
+          <t>Design of Digital Platforms</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Advanced Network Control and Management</t>
+          <t>Introduction to Data Science Tools</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Finance for Science and Technology Students</t>
+          <t>Design of Cyber-Physical Systems</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Applied Project Management</t>
+          <t>Analog and Mixed-Signal Electronics for Signal Processing</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Applied Cryptography and Network Security</t>
+          <t>Machine learning and natural language processing</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Intrusion Detection in Physical and Virtual Networks</t>
+          <t>GPU Programming</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Introduction to Data Privacy</t>
+          <t>Information Technology Security Methods</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Dependable Performance Design</t>
+          <t>CRITICAL INFRASTRUCTURES FOR INNOVATIVE POWER DISTRIBUTION</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Design of Cyber-Physical Systems</t>
+          <t>Machine Learning Applied to Security</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Advanced Internet Technologies - Networked Systems, Specialization Course</t>
+          <t>Cryptography</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Distributed Systems</t>
+          <t>INTRODUCTION TO SOFTWARE DEVELOPMENT</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Quantum Cryptography</t>
+          <t>Discrete mathematics</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Time Series Analysis</t>
+          <t>5G Mobile Networks, Technologies &amp; Security</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Performance analysis of computer systems</t>
+          <t>Mobile Networks</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>From an Idea to Reality</t>
+          <t>AUTOMATED REASONING</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Network Measurements and Analysis</t>
+          <t>Development of Secure Software</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Machine Learning</t>
+          <t>Introduction to Computer Networks</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Machine Learning for Earth Observation powered by Supercomputers</t>
+          <t>Identification, Authentication and Authorization</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Programming Projects on Internet of Things</t>
+          <t>Analysis</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Introduction to deep neural networks</t>
+          <t>Operating System &amp; Architecture</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>Introduction to Design Thinking</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Software Testing</t>
+          <t>Dependable Performance Design</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Fundaments of the Internet</t>
+          <t>Cryptology &amp; Applications</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Reasoned Programming</t>
+          <t>Advanced Computer Networking</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Biometric security systems</t>
+          <t>DISTRIBUTED SYSTEMS</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Foreign language in science and technology</t>
+          <t>Embedded Security Assessment</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Introduction to cryptography</t>
+          <t>DEEP LEARNING</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Fighting crime in cyberspace and legal aspects of cybersecurity</t>
+          <t xml:space="preserve">Formal Methods for Software Analysis </t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Security of IoT systems</t>
+          <t>Information theory</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Security and safety in control systems and industrial networks</t>
+          <t>System Development in C#/.NET</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>History of ideas and scientific discoveries</t>
+          <t>Stochastic Signal and System Analysis</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Quantum cryptography</t>
+          <t>Fundaments of Cryptography</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Mathematical foundations of cryptography</t>
+          <t>Communication Systems for IoT</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Information society</t>
+          <t>FOUNDATIONS OF LEGAL SYSTEM AND STATE ORGANISATION</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Cryptography and Network Security</t>
+          <t>Machine Learning, Advanced Course</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Digital Signal Processing for Communications and Information Systems</t>
+          <t>Advanced Cryptographic and Security Technologies (Blockchain technologies)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Analog and Mixed-Signal Electronics for Signal Processing</t>
+          <t>Basic General Algebra</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Analysis of Digital Communication Systems</t>
+          <t>Introduction to deep neural networks</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Building Blocks for Telecom Systems</t>
+          <t>Biometric Systems</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Design of Digital Platforms</t>
+          <t>TECHNICAL SECURITY</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Computer Architectures</t>
+          <t>VERIFICATION AND VALIDATION TECHNIQUES IN AI AND CYBERSECURITY</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Stochastic Signal and System Analysis</t>
+          <t>Malware Analysis Methods</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Electromagnetic Propagation</t>
+          <t>Software Testing</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Mobile Networks</t>
+          <t>ICT Law II</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Hardware Security</t>
+          <t>Distributed Systems</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Telecommunications and Security Management</t>
+          <t>Programming fundamentals</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Privacy Technologies</t>
+          <t>Correcting codes</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>e-Security</t>
+          <t>Automobile Electric and Electronic Systems</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Software for Real-Time Control</t>
+          <t>Computer Networks - practicals</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>6G Communication Networks</t>
+          <t>Security of IoT systems</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Distributed Systems</t>
+          <t>Electrical Engineering 1</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Advanced Methods in Cryptography</t>
+          <t>Access and Transport Networks</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Image Analysis and Understanding</t>
+          <t>Advanced algebraic structures</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Satellite Navigation and Communications</t>
+          <t>Fundaments of the Internet</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Multimedia Technology and Coding</t>
+          <t>Introduction to Quantum Computer Programming</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Philosophy of Technology</t>
+          <t>Quantum cryptography</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Engineering Economy</t>
+          <t>Blockchain principles and applications</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Introduction to Safety Engineering</t>
+          <t>Intrusion Detection in Physical and Virtual Networks</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Total Quality Management</t>
+          <t>Operating Systems and System Programming</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Intellectual Property Management</t>
+          <t>Registration for SB200</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>New and Emerging Technologies</t>
+          <t>Verification of security protocols</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Robotics Applications</t>
+          <t>Cyber Warfare</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Data Science Applications II</t>
+          <t>Foundations of Machine Learning</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Basic General Algebra</t>
+          <t>Multimedia Technology and Coding</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Basic algorithms</t>
+          <t>Machine Learning &amp; AI for Security</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Information theory</t>
+          <t>Elliptic Curves for Cryptography</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Correcting codes</t>
+          <t>Data protection, Privacy and Anonymity</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Complexity</t>
+          <t>Analysis of Digital Communication Systems</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Biometric security systems</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Elliptic Curves for Cryptography</t>
+          <t>DEEP LEARNING FUNDAMENTALS</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Cryptanalysis</t>
+          <t>UNIX</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Software Security</t>
+          <t>Design of Fault-tolerant Systems</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Euclidean networks in cryptography</t>
+          <t>Dependability and Performance with Discrete Event Simulation</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Blockchain principles and applications</t>
+          <t>System administration - Databases</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Parallel programming, GPU</t>
+          <t>Script programming</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Protocol Security</t>
+          <t>OPERATING SYSTEMS</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Correcting codes in cryptography</t>
+          <t>Foundations of Programming</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Quantum Cryptography</t>
+          <t>BASICS OF SOCIOLOGY FOR CRIMINAL JUSTICE PROFESSIONALS</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Algorithmic number theory for cryptography</t>
+          <t>Information society</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Big Data Infrastructures</t>
+          <t>Digital Signal Processing for Communications and Information Systems</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Open-Source Intelligence</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Basic Network Security</t>
+          <t>Advanced Topics in Networking</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t xml:space="preserve">Data security and protection
+</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Machine Learning &amp; AI for Security</t>
+          <t>ECONOMIC CRIME</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Mobile Network Security</t>
+          <t>Computer Architectures</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Embedded Security Assessment</t>
+          <t>Advanced Methods in Cryptography</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cryptology </t>
+          <t>Machine Learning</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Cyberattacks Crime and Defenses</t>
+          <t>STOCHASTIC MODELS</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Advanced Network Security</t>
+          <t>Time Series Analysis</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Physical aspects of digital security</t>
+          <t>Reasoned Programming</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Verification of security protocols</t>
+          <t>Image Analysis and Understanding</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Cryptographic protocols</t>
+          <t>Application of Machine Learning in Information Security</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Applied cryptography</t>
+          <t>PHYSICAL-LAYER TECHNIQUES FOR WIRELESS COMMUNICATION SECURITY</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Advanced algorithms</t>
+          <t>Software Security</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Intrusion Detection Laboratory</t>
+          <t>Applied cryptography</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CRYPTOGRAPHY</t>
+          <t>Computer Systems</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>DEEP LEARNING FUNDAMENTALS</t>
+          <t>Theoretical Informatics</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>MACHINE LEARNING APPLIED TO CYBERSECURITY AND CYBERCRIME</t>
+          <t>Processing of Structured Documents</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>AUTHENTICATION TECHNOLOGIES</t>
+          <t>Mobile Network Security</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Algorithms &amp; Data Structures</t>
+          <t>Machine Learning in Image Processing</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Introduction to Data Privacy</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Discrete mathematics</t>
+          <t>Network security</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Cryptology &amp; Applications</t>
+          <t>Data Science</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Networking I</t>
+          <t>Television Technology and Multimedia</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>object oriented programing</t>
+          <t>Mobile Communication</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Operating System &amp; Architecture</t>
+          <t>Network design - Wireless networks</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>5G Mobile Networks, Technologies &amp; Security</t>
+          <t>Algorithms &amp; Data Structures</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Network Defense &amp; Architecture</t>
+          <t>Hardware &amp; Wireless Security (Hardware and embedded security)</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Networks &amp; Cloud Technologies and Security (Computer networks and cloud technologies)</t>
+          <t>Data Analytics and Machine Learning</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Networks &amp; Cloud Technologies and Security (Network and Cloud Security)</t>
+          <t>German/Macedonian</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Cryptography</t>
+          <t>Hardware of Computer Networks</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Hardware &amp; Wireless Security (Hardware and embedded security)</t>
+          <t>Computers and Programming 1</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Hardware &amp; Wireless Security (Wireless and device-to-device communication Security)</t>
+          <t>Philosophy of Technology</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Web Applications</t>
+          <t>Applied Cryptography</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Advanced cryptography</t>
+          <t>Physical aspects of digital security</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>AI and Cybersecurity</t>
+          <t>Mathematical Foundations of Computer Science</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Data protection, Privacy and Anonymity</t>
+          <t>Basic algorithms</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Post-Quantum Cryptography</t>
+          <t>Advanced Algorithms</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Network design - Introduction</t>
+          <t>ADVANCED ALGORITHMS</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>System administration - Introduction</t>
+          <t>Authentication and Access Control</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Network design - Switching and Routing</t>
+          <t>Operating Systems and Virtualization</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Network design - WAN and operator networks</t>
+          <t>Parallel programming, GPU</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Network security</t>
+          <t>Data Communication</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Network design - Wireless networks</t>
+          <t>NETWORKED CONTROL SYSTEMS AND SECURITY</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Script programming</t>
+          <t>Security Technologies</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>System administration - Databases</t>
+          <t>Foundations of Object Oriented Programming in Java</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>AUTOMATED REASONING</t>
+          <t>Mathematical Logic for Computer Science</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>DEEP LEARNING</t>
+          <t>From an Idea to Reality</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>VERIFICATION AND VALIDATION TECHNIQUES IN AI AND CYBERSECURITY</t>
+          <t>Intellectual Property Management</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>ADVANCED ALGORITHMS</t>
+          <t>Secure Communications</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>ADVANCED DATA SCIENCE</t>
+          <t>Design Seminar for Digital Platforms</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>ADVANCED DATABASE SYSTEMS</t>
+          <t>Applied Mathematics Complements</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>AUDITORY AND TACTILE INTERACTIONS</t>
+          <t>Performance analysis of computer systems</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>COMPUTER VISION</t>
+          <t>SUPERVISORY CONTROL AND MONITORING</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>DISTRIBUTED SYSTEMS</t>
+          <t>6G Communication Networks</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>FORMAL METHODS FOR SECURITY</t>
+          <t>Python</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>FOUNDATIONS OF NEURAL NETWORKS</t>
+          <t>Multimedia Services</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>GENERATIVE AI</t>
+          <t>Advanced cryptography</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>INFORMATION RETRIEVAL</t>
+          <t>ADVANCED EMBEDDED SYSTEMS</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>QUANTUM COMPUTING AND COMMUNICATION</t>
+          <t>Applied Information Theory</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Communication Technology</t>
+          <t>CRYPTOGRAPHY</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Computers and Programming 1</t>
+          <t>Statistics and Probabilities</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Legal Theory</t>
+          <t>Computer Networks</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Foundations of Cryptography</t>
+          <t>Network Measurements and Analysis</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>System administration - Introduction</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Computers and Programming 2</t>
+          <t>The C++ Programming Language</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Fundamentals of Information and Communication Technologies</t>
+          <t>INTERNET OF THINGS</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Data Communication</t>
+          <t>VIOLENCE AND SOCIETY</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Theoretical Informatics</t>
+          <t>Engineering Economy</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>ICT Security 2</t>
+          <t>Research Methods and Scientific Ethics</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Multimedia Services</t>
+          <t>INFORMATION RETRIEVAL</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Electrical Engineering 1</t>
+          <t>Total Quality Management</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Access and Transport Networks</t>
+          <t>Foreign language in science and technology</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Security Systems</t>
+          <t>Building Blocks for Telecom Systems</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Introduction to Computer Typography and Graphics</t>
+          <t>Cryptographic Protocols</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Network Architecture</t>
+          <t>Telecommunications and Security Management</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Digital Electronics 1</t>
+          <t>Laboratory of security and applied cryptography</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Hardware of Computer Networks</t>
+          <t>Basic Network Security</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Communication Systems for IoT</t>
+          <t>Communication Technology</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Mobile Communication</t>
+          <t>Computer Networks and Security</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Object-Oriented Programming</t>
+          <t>FAULT DIAGNOSIS AND ESTIMATION IN DYNAMICAL</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Transmission Media</t>
+          <t>Computer Modeling of Electrical Devices and Components</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>The C++ Programming Language</t>
+          <t>Legal Theory</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Analog Technology</t>
+          <t>Network Security</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Automobile Electric and Electronic Systems</t>
+          <t>AUTHENTICATION TECHNOLOGIES</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Computer Modeling of Electrical Devices and Components</t>
+          <t>MACHINE LEARNING</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Television Technology and Multimedia</t>
+          <t>Mathematical foundations of cryptography</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Artificial Intelligence</t>
+          <t>Operating Systems</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Introduction to Programming Systems</t>
+          <t>Introduction to Safety Engineering</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Data Science</t>
+          <t>Network design - WAN and operator networks</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Privacy &amp; Cryptography</t>
+          <t>Artificial Neural Networks and Deep Architectures</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>Web Applications</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Network Security</t>
+          <t>Object-Oriented Programming</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Malware Analysis</t>
+          <t>Coding Theory and Applications</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Cryptography and Network Security</t>
+          <t>BIOMETRIC TECHNOLOGIES AND BEHAVIOURAL SECURITY</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Cryptographic Protocols</t>
+          <t>Advanced Network Security</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Advanced Methods in Cryptography</t>
+          <t>Statistical Methods in Applied Computer Science</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Privacy Technologies</t>
+          <t>Software Safety and Security</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Advanced Privacy Technologies</t>
+          <t>Data Science Applications II</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Design of Digital Platforms</t>
+          <t>INDUSTRIAL SOFTWARE DEVELOPMENT</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Design Seminar for Digital Platforms</t>
+          <t>History of ideas and scientific discoveries</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Hardware Security</t>
+          <t>Software Reverse Engineering</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Development of Secure Software</t>
+          <t>Artificial Intelligence</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Security and Privacy in Contemporary Distributed Software Systems</t>
+          <t>Database Systems</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Practical Cryptography</t>
+          <t>Correcting codes in cryptography</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>Degree Project in Computer Science and Engineering, specialising in Cybersecurity</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Fraud Detection</t>
+          <t>Complexity</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Processing of Structured Documents</t>
+          <t>Reinforcement Learning</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Big Data and Cloud Computing</t>
+          <t>QUANTUM COMPUTING AND COMMUNICATION</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Advanced Topics in Databases</t>
+          <t>PRIVATE SECURITY AND PRIVATE DETECTIVE ACTIVITY</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Advanced Topics in Networking</t>
+          <t>AUDITORY AND TACTILE INTERACTIONS</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Network Security</t>
+          <t>Transmission Media</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data security and protection
-</t>
+          <t>Applied Project Management</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>FAULT DIAGNOSIS AND ESTIMATION IN DYNAMICAL</t>
+          <t>Scripting Languages</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>INDUSTRIAL SOFTWARE DEVELOPMENT</t>
+          <t>ADVANCED DATA SCIENCE</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>MACHINE LEARNING</t>
+          <t>Post-Quantum Cryptography</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>ARTIFICIAL INTELLIGENCE</t>
+          <t>Introduction to Computer Typography and Graphics</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>OPERATING SYSTEMS</t>
+          <t>Machine Learning for Earth Observation powered by Supercomputers</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>SUPERVISORY CONTROL AND MONITORING</t>
+          <t>Software for Real-Time Control</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>DATA DRIVEN MODELS FOR SYSTEM ENGINEERING</t>
+          <t>Electromagnetic Propagation</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>CRITICAL INFRASTRUCTURES FOR INNOVATIVE POWER DISTRIBUTION</t>
+          <t>Introduction to cryptography</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>INTERNET OF THINGS</t>
+          <t>Statistics for Computer Science</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>ADVANCED EMBEDDED SYSTEMS</t>
+          <t>Algorithmic number theory for cryptography</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>NETWORKED CONTROL SYSTEMS AND SECURITY</t>
+          <t>Pros and Cons of Intelligent Systems</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>STOCHASTIC MODELS</t>
+          <t>Advanced Network Control and Management</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>PHYSICAL-LAYER TECHNIQUES FOR WIRELESS COMMUNICATION SECURITY</t>
+          <t>Fraud Detection</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>BIOMETRIC TECHNOLOGIES AND BEHAVIOURAL SECURITY</t>
+          <t>Random processes</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Secure Communications</t>
+          <t>Advanced algorithms</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Software Reverse Engineering</t>
+          <t>Network design - Switching and Routing</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Laboratory of security and applied cryptography</t>
+          <t>Advanced Topics in Databases</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Security Technologies</t>
+          <t>Big Data Infrastructures</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Advanced Topics in Information Technology Security</t>
+          <t>Intrusion Detection Laboratory</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Machine learning and natural language processing</t>
+          <t>Network design - Introduction</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Machine Learning in Image Processing</t>
+          <t>Introduction to IoT</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>System Development in C#/.NET</t>
+          <t>CRIMINAL LAW SYSTEM OF REPUBLIC OF SLOVENIA</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>GPU Programming</t>
+          <t>Cryptography and Network Security</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Python Seminar</t>
+          <t>Euclidean networks in cryptography</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Introduction to Quantum Computer Programming</t>
+          <t>Malware Analysis</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Introduction to IoT</t>
+          <t>DATA DRIVEN MODELS FOR SYSTEM ENGINEERING</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Privacy &amp; Cryptography</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Fundaments of Cryptography</t>
+          <t>Finance for Science and Technology Students</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Probability in Computer Science</t>
+          <t>Networks &amp; Cloud Technologies and Security (Computer networks and cloud technologies)</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Advanced Computer Networking</t>
+          <t>Aplicated math</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Statistics for Computer Science</t>
+          <t>Big Data and Cloud Computing</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t xml:space="preserve">Formal Methods for Software Analysis </t>
+          <t>FORMAL METHODS FOR SECURITY</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Advanced Topics in Information Technology Security</t>
+          <t>Network Defense &amp; Architecture</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Mathematical Foundations of Computer Science</t>
+          <t>Biometrics</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Foundations of Programming</t>
+          <t>Introduction to Programming Systems</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Computer Systems</t>
+          <t>AI and Cybersecurity</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>Database Systems</t>
+          <t>Cyberattacks Crime and Defenses</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Introduction to Programming and Algorithms II</t>
+          <t>Hardware Security</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>Principles of low-level programming</t>
+          <t>INTRODUCTION TO CRIMINOLOGY WITH PENOLOGY</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Operating Systems</t>
+          <t>Networking I</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>Computer Networks</t>
+          <t>Cryptanalysis</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Computer Networks - practicals</t>
+          <t>e-Security</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>UNIX</t>
+          <t>NATIONAL SECURITY SYSTEM</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>ICT Law II</t>
+          <t>Security Systems</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Cyber Warfare</t>
+          <t>ADVANCED DATABASE SYSTEMS</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Introduction to Informatics</t>
+          <t>object oriented programing</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Pros and Cons of Intelligent Systems</t>
+          <t>Advanced Information Security</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Linear algebra and discrete mathematics</t>
+          <t>Python Seminar</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Foundations of Object Oriented Programming in Java</t>
+          <t>Electronic Document Preparation</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Registration for SB200</t>
+          <t>Quantum Cryptography</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Authentication and Access Control</t>
+          <t>Security and Privacy in Contemporary Distributed Software Systems</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Electronic Document Preparation</t>
+          <t xml:space="preserve">Cryptology </t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>Advanced Internet Technologies - Networked Systems, Specialization Course</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Foundations of Cryptography</t>
+          <t>Fundamentals of Information and Communication Technologies</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Cyber-Physical Security in Time-Critical Systems</t>
+          <t>Cryptographic Systems</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Design of Fault-tolerant Systems</t>
+          <t>New and Emerging Technologies</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Hardware Security</t>
+          <t>Analog Technology</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Foundations of Machine Learning</t>
+          <t>Protocol Security</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Machine Learning</t>
+          <t>ARTIFICIAL INTELLIGENCE</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Machine Learning, Advanced Course</t>
+          <t>Networks &amp; Cloud Technologies and Security (Network and Cloud Security)</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Artificial Neural Networks and Deep Architectures</t>
+          <t>MACHINE LEARNING APPLIED TO CYBERSECURITY AND CYBERCRIME</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Advanced Algorithms</t>
+          <t>Cryptographic Engineering</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Parallel and Distributed Computing</t>
+          <t>Cyber-Physical Security in Time-Critical Systems</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Statistical Methods in Applied Computer Science</t>
+          <t>FOUNDATIONS OF NEURAL NETWORKS</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Reinforcement Learning</t>
+          <t>Digital Electronics 1</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Degree Project in Computer Science and Engineering, specialising in Cybersecurity</t>
+          <t>ICT Security 2</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Software Safety and Security</t>
+          <t>Hardware &amp; Wireless Security (Wireless and device-to-device communication Security)</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Applied Cryptography</t>
+          <t>Network and Communications Security</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Biometrics</t>
+          <t>Network Architecture</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Machine Learning Applied to Security</t>
+          <t>Algorithms and Data Structures</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Identification, Authentication and Authorization</t>
+          <t>Security and safety in control systems and industrial networks</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Quantum Security</t>
-        </is>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" t="inlineStr">
-        <is>
-          <t>Information Technology Security Methods</t>
-        </is>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" t="inlineStr">
-        <is>
-          <t>Cryptographic Systems</t>
-        </is>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" t="inlineStr">
-        <is>
-          <t>Malware Analysis Methods</t>
-        </is>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" t="inlineStr">
-        <is>
-          <t>FOUNDATIONS OF LEGAL SYSTEM AND STATE ORGANISATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" t="inlineStr">
-        <is>
-          <t>NATIONAL SECURITY SYSTEM</t>
-        </is>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" t="inlineStr">
-        <is>
-          <t>INTRODUCTION TO SOFTWARE DEVELOPMENT</t>
-        </is>
-      </c>
-    </row>
-    <row r="296">
-      <c r="A296" t="inlineStr">
-        <is>
-          <t>BASICS OF SOCIOLOGY FOR CRIMINAL JUSTICE PROFESSIONALS</t>
-        </is>
-      </c>
-    </row>
-    <row r="297">
-      <c r="A297" t="inlineStr">
-        <is>
-          <t>INTRODUCTION TO CRIMINOLOGY WITH PENOLOGY</t>
-        </is>
-      </c>
-    </row>
-    <row r="298">
-      <c r="A298" t="inlineStr">
-        <is>
-          <t>CRIMINAL LAW SYSTEM OF REPUBLIC OF SLOVENIA</t>
-        </is>
-      </c>
-    </row>
-    <row r="299">
-      <c r="A299" t="inlineStr">
-        <is>
-          <t>CRIMINAL JUSTICE AND SECURITY TERMINOLOGY IN ENGLISH</t>
-        </is>
-      </c>
-    </row>
-    <row r="300">
-      <c r="A300" t="inlineStr">
-        <is>
-          <t>TECHNICAL SECURITY</t>
-        </is>
-      </c>
-    </row>
-    <row r="301">
-      <c r="A301" t="inlineStr">
-        <is>
-          <t>ECONOMIC CRIME</t>
-        </is>
-      </c>
-    </row>
-    <row r="302">
-      <c r="A302" t="inlineStr">
-        <is>
-          <t>PRIVATE SECURITY AND PRIVATE DETECTIVE ACTIVITY</t>
-        </is>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" t="inlineStr">
-        <is>
-          <t>VIOLENCE AND SOCIETY</t>
-        </is>
-      </c>
-    </row>
-    <row r="304">
-      <c r="A304" t="inlineStr">
-        <is>
-          <t>Network and Communications Security</t>
-        </is>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" t="inlineStr">
-        <is>
-          <t>Data Analytics and Machine Learning</t>
-        </is>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="inlineStr">
-        <is>
-          <t>Applied Cryptography</t>
-        </is>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" t="inlineStr">
-        <is>
-          <t>Advanced Cryptographic and Security Technologies (Blockchain technologies)</t>
-        </is>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" t="inlineStr">
-        <is>
-          <t>Programming fundamentals</t>
-        </is>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" t="inlineStr">
-        <is>
-          <t>Aplicated math</t>
-        </is>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" t="inlineStr">
-        <is>
-          <t>Operating Systems and Virtualization</t>
-        </is>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" t="inlineStr">
-        <is>
-          <t>Algorithms and Data Structures</t>
-        </is>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" t="inlineStr">
-        <is>
-          <t>Applied Mathematics Complements</t>
-        </is>
-      </c>
-    </row>
-    <row r="313">
-      <c r="A313" t="inlineStr">
-        <is>
-          <t>Introduction to Computer Networks</t>
-        </is>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" t="inlineStr">
-        <is>
-          <t>Introduction to Design Thinking</t>
-        </is>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" t="inlineStr">
-        <is>
-          <t>Statistics and Probabilities</t>
-        </is>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" t="inlineStr">
-        <is>
-          <t>Applied Cryptography</t>
+          <t>Satellite Navigation and Communications</t>
         </is>
       </c>
     </row>

</xml_diff>